<commit_message>
[Fix] : TrainSkill 누락된거 수정
</commit_message>
<xml_diff>
--- a/Assets/02_Resources/Data/ChoiceData.xlsx
+++ b/Assets/02_Resources/Data/ChoiceData.xlsx
@@ -1,21 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="HCell" lastEdited="11.0" lowestEdited="11.0" rupBuild="0.2292"/>
-  <workbookPr codeName="ThisWorkbook" autoCompressPictures="1"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="28545" windowHeight="11700"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200"/>
   </bookViews>
   <sheets>
-    <sheet name="Add_Train_Choice_Data" sheetId="1" r:id="rId4"/>
-    <sheet name="Upgrade_Train_Choice_Data" sheetId="2" r:id="rId5"/>
+    <sheet name="Add_Train_Choice_Data" sheetId="1" r:id="rId1"/>
+    <sheet name="Upgrade_Train_Choice_Data" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr/>
+  <fileRecoveryPr autoRecover="0" crashSave="0" dataExtractLoad="0" repairLoad="1"/>
+  <extLst>
+    <ext uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="8">
   <si>
     <t xml:space="preserve">train_data_id</t>
   </si>
@@ -46,36 +52,17 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="맑은 고딕"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
+      <sz val="8"/>
+      <name val="돋움"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
   </fonts>
   <fills count="2">
@@ -88,18 +75,11 @@
   </fills>
   <borders count="4">
     <border>
-      <left>
-        <color indexed="64"/>
-      </left>
-      <right>
-        <color indexed="64"/>
-      </right>
-      <top>
-        <color indexed="64"/>
-      </top>
-      <bottom>
-        <color indexed="64"/>
-      </bottom>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="medium">
@@ -111,9 +91,8 @@
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom>
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="medium">
@@ -122,12 +101,9 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top>
-        <color indexed="64"/>
-      </top>
-      <bottom>
-        <color indexed="64"/>
-      </bottom>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="medium">
@@ -136,12 +112,11 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top>
-        <color indexed="64"/>
-      </top>
+      <top/>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -153,9 +128,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -179,10 +152,41 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf/>
+  <dxfs count="7">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFAEBFEA"/>
+          <bgColor rgb="FFAEBFEA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFAEBFEA"/>
+          <bgColor rgb="FFAEBFEA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF94A5DF"/>
+          <bgColor rgb="FF94A5DF"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color rgb="FF6182D6"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF6182D6"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -215,30 +219,36 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF6182D6"/>
+          <bgColor rgb="FF6182D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="Normal Style 1 - Accent 1" pivot="0" table="1" count="9">
-      <tableStyleElement type="wholeTable" size="1"/>
-      <tableStyleElement type="headerRow" size="1" dxfId="5"/>
-      <tableStyleElement type="totalRow" size="1" dxfId="4"/>
-      <tableStyleElement type="firstColumn" size="1" dxfId="3"/>
-      <tableStyleElement type="lastColumn" size="1" dxfId="3"/>
-      <tableStyleElement type="firstRowStripe" size="1" dxfId="2"/>
-      <tableStyleElement type="secondRowStripe" size="1" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" size="1" dxfId="2"/>
-      <tableStyleElement type="secondColumnStripe" size="1" dxfId="1"/>
+    <tableStyle name="Normal Style 1 - Accent 1" pivot="0" table="0" count="6">
+      <tableStyleElement type="firstColumn" dxfId="6"/>
+      <tableStyleElement type="lastColumn" dxfId="5"/>
+      <tableStyleElement type="firstRowStripe" dxfId="4"/>
+      <tableStyleElement type="secondRowStripe" dxfId="3"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="2"/>
+      <tableStyleElement type="secondColumnStripe" dxfId="1"/>
     </tableStyle>
-    <tableStyle name="Light Style 1 - Accent 1" pivot="1" table="0" count="8">
-      <tableStyleElement type="wholeTable" size="1" dxfId="6"/>
-      <tableStyleElement type="headerRow" size="1" dxfId="11"/>
-      <tableStyleElement type="totalRow" size="1" dxfId="10"/>
-      <tableStyleElement type="firstColumn" size="1" dxfId="9"/>
-      <tableStyleElement type="lastColumn" size="1" dxfId="9"/>
-      <tableStyleElement type="firstRowStripe" size="1" dxfId="7"/>
-      <tableStyleElement type="secondRowStripe" size="1" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" size="1" dxfId="8"/>
+    <tableStyle name="Light Style 1 - Accent 1" pivot="0" table="0" count="1">
+      <tableStyleElement type="secondRowStripe"/>
     </tableStyle>
   </tableStyles>
+  <extLst>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -520,6 +530,8 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -527,9 +539,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:F19"/>
-  <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="16.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
-    <col min="1" max="1" width="9.00390625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" style="1" customWidth="1"/>
     <col min="3" max="3" width="12.640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="14.28515625" style="1" customWidth="1"/>
@@ -538,7 +550,7 @@
     <col min="7" max="7" width="13.92578125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -555,7 +567,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="16.75" customHeight="1">
+    <row r="2" spans="1:5" ht="16.75" customHeight="1" x14ac:dyDescent="0.55">
       <c r="A2" s="3">
         <v>60001</v>
       </c>
@@ -569,7 +581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A3" s="4">
         <v>60002</v>
       </c>
@@ -583,7 +595,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A4" s="4">
         <v>60003</v>
       </c>
@@ -597,7 +609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A5" s="4">
         <v>60004</v>
       </c>
@@ -611,7 +623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A6" s="4">
         <v>60005</v>
       </c>
@@ -625,7 +637,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A7" s="4">
         <v>60006</v>
       </c>
@@ -639,7 +651,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A8" s="4">
         <v>60007</v>
       </c>
@@ -653,7 +665,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A9" s="4">
         <v>60008</v>
       </c>
@@ -667,7 +679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A10" s="5">
         <v>60009</v>
       </c>
@@ -681,7 +693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A11" s="6">
         <v>61001</v>
       </c>
@@ -695,7 +707,7 @@
         <v>30001</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A12" s="7">
         <v>61002</v>
       </c>
@@ -709,7 +721,7 @@
         <v>30002</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A13" s="7">
         <v>61003</v>
       </c>
@@ -723,7 +735,7 @@
         <v>30003</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A14" s="7">
         <v>61004</v>
       </c>
@@ -737,7 +749,7 @@
         <v>30004</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A15" s="7">
         <v>61005</v>
       </c>
@@ -751,7 +763,7 @@
         <v>30005</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A16" s="7">
         <v>61006</v>
       </c>
@@ -765,7 +777,7 @@
         <v>30006</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A17" s="7">
         <v>61007</v>
       </c>
@@ -779,7 +791,7 @@
         <v>30007</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A18" s="7">
         <v>61008</v>
       </c>
@@ -793,7 +805,7 @@
         <v>40001</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A19" s="8">
         <v>61009</v>
       </c>
@@ -808,8 +820,9 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait"/>
+  <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -817,7 +830,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:F16"/>
-  <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="16.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="1" max="1" width="10" style="1" customWidth="1"/>
     <col min="2" max="2" width="13.92578125" style="1" customWidth="1"/>
@@ -826,7 +839,7 @@
     <col min="5" max="5" width="13.78515625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -843,7 +856,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="16.75" customHeight="1">
+    <row r="2" spans="1:5" ht="16.75" customHeight="1" x14ac:dyDescent="0.55">
       <c r="A2" s="3">
         <v>70001</v>
       </c>
@@ -860,7 +873,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A3" s="4">
         <v>70002</v>
       </c>
@@ -877,7 +890,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A4" s="4">
         <v>70003</v>
       </c>
@@ -894,7 +907,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A5" s="4">
         <v>70004</v>
       </c>
@@ -911,7 +924,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A6" s="4">
         <v>70005</v>
       </c>
@@ -928,7 +941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A7" s="4">
         <v>70006</v>
       </c>
@@ -945,7 +958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A8" s="4">
         <v>70007</v>
       </c>
@@ -962,7 +975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A9" s="4">
         <v>70008</v>
       </c>
@@ -979,7 +992,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A10" s="4">
         <v>70009</v>
       </c>
@@ -996,25 +1009,26 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:1">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A11" s="4"/>
     </row>
-    <row r="12" spans="1:1">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A12" s="4"/>
     </row>
-    <row r="13" spans="1:1">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A13" s="4"/>
     </row>
-    <row r="14" spans="1:1">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A14" s="4"/>
     </row>
-    <row r="15" spans="1:1">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A15" s="4"/>
     </row>
-    <row r="16" spans="1:1" ht="16.75" customHeight="1">
+    <row r="16" spans="1:5" ht="16.75" customHeight="1" x14ac:dyDescent="0.55">
       <c r="A16" s="5"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait"/>
 </worksheet>

</xml_diff>

<commit_message>
[Add] 엘리트 트레인 trainSkillDataIds / passiveSkillDataIds 설정
- TrainData.xlsx: 31001/31005/31006/42001/42002 H열(trainSkill) 추가
  - DB.asset: 동일 5개 trainSkillDataIds 배열 설정
  - passiveSkillDataIds(60001-60009)는 이미 세팅된 상태 확인
</commit_message>
<xml_diff>
--- a/Assets/02_Resources/Data/ChoiceData.xlsx
+++ b/Assets/02_Resources/Data/ChoiceData.xlsx
@@ -1,52 +1,55 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="28545" windowHeight="11700" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView windowWidth="28545" windowHeight="11700" tabRatio="600"/>
   </bookViews>
   <sheets>
-    <sheet name="Add_Train_Choice_Data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Upgrade_Train_Choice_Data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Add_Train_Choice_Data" sheetId="1" r:id="rId1"/>
+    <sheet name="Upgrade_Train_Choice_Data" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="0" uniqueCount="0"/>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
   <fonts count="6">
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="맑은 고딕"/>
-      <color rgb="FF000000"/>
-      <sz val="11"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="맑은 고딕"/>
-      <color rgb="FF000000"/>
-      <sz val="11"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="맑은 고딕"/>
-      <color rgb="FF000000"/>
-      <sz val="11"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="맑은 고딕"/>
-      <color rgb="FF000000"/>
-      <sz val="11"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="맑은 고딕"/>
-      <color rgb="FF000000"/>
-      <sz val="11"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="맑은 고딕"/>
-      <color rgb="FF000000"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -121,32 +124,32 @@
     </xf>
   </cellStyleXfs>
   <cellXfs count="10">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -564,475 +567,791 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet1">
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.4"/>
   <cols>
-    <col width="13.29296875" bestFit="1" customWidth="1" style="3" min="1" max="1"/>
-    <col width="12" customWidth="1" style="2" min="2" max="2"/>
-    <col width="12.640625" customWidth="1" style="2" min="3" max="3"/>
-    <col width="14.28515625" customWidth="1" style="2" min="4" max="4"/>
-    <col width="16.92578125" customWidth="1" style="2" min="5" max="5"/>
-    <col width="20" customWidth="1" style="2" min="6" max="6"/>
-    <col width="13.92578125" customWidth="1" style="2" min="7" max="7"/>
+    <col min="1" max="1" width="13.29296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" style="2" customWidth="1"/>
+    <col min="3" max="3" width="12.640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="16.92578125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="20" style="2" customWidth="1"/>
+    <col min="7" max="7" width="13.92578125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>id</t>
+        <v>id</v>
+        <is>
+          <t xml:space="preserve">id</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>train_data_id</t>
+        <v>train_data_id</v>
+        <is>
+          <t xml:space="preserve">train_data_id</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>weight</t>
+        <v>weight</v>
+        <is>
+          <t xml:space="preserve">weight</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>tier</t>
+        <v>tier</v>
+        <is>
+          <t xml:space="preserve">tier</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>replace_train_id</t>
+        <v>replace_train_id</v>
+        <is>
+          <t xml:space="preserve">replace_train_id</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>skill_type</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="16.75" customHeight="1" s="2">
-      <c r="A2" s="7" t="n">
+        <v>skill_type</v>
+        <is>
+          <t xml:space="preserve">skill_type</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" s="2" ht="16.75" customHeight="1">
+      <c r="A2" s="7">
         <v>60001</v>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="3">
         <v>30001</v>
       </c>
-      <c r="C2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" s="3" t="n">
+      <c r="C2" s="3">
+        <v>0</v>
+      </c>
+      <c r="D2" s="3">
+        <v>0</v>
+      </c>
+      <c r="F2" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="n">
+      <c r="A3" s="8">
         <v>60002</v>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="3">
         <v>30002</v>
       </c>
-      <c r="C3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="3" t="n">
+      <c r="C3" s="3">
+        <v>0</v>
+      </c>
+      <c r="D3" s="3">
+        <v>0</v>
+      </c>
+      <c r="F3" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="n">
+      <c r="A4" s="8">
         <v>60003</v>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="3">
         <v>30003</v>
       </c>
-      <c r="C4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="3" t="n">
+      <c r="C4" s="3">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="n">
+      <c r="A5" s="8">
         <v>60004</v>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="3">
         <v>30004</v>
       </c>
-      <c r="C5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="3" t="n">
+      <c r="C5" s="3">
+        <v>0</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0</v>
+      </c>
+      <c r="F5" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="n">
+      <c r="A6" s="8">
         <v>60005</v>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="3">
         <v>30005</v>
       </c>
-      <c r="C6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="3" t="n">
+      <c r="C6" s="3">
+        <v>0</v>
+      </c>
+      <c r="D6" s="3">
+        <v>0</v>
+      </c>
+      <c r="F6" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n">
+      <c r="A7" s="8">
         <v>60006</v>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" s="3">
         <v>30006</v>
       </c>
-      <c r="C7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="3" t="n">
+      <c r="C7" s="3">
+        <v>0</v>
+      </c>
+      <c r="D7" s="3">
+        <v>0</v>
+      </c>
+      <c r="F7" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="n">
+      <c r="A8" s="8">
         <v>60007</v>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" s="3">
         <v>30007</v>
       </c>
-      <c r="C8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="3" t="n">
+      <c r="C8" s="3">
+        <v>0</v>
+      </c>
+      <c r="D8" s="3">
+        <v>0</v>
+      </c>
+      <c r="F8" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="n">
+      <c r="A9" s="8">
         <v>60008</v>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B9" s="3">
         <v>40001</v>
       </c>
-      <c r="C9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" ht="16.75" customHeight="1" s="2">
-      <c r="A10" s="9" t="n">
+      <c r="C9" s="3">
+        <v>0</v>
+      </c>
+      <c r="D9" s="3">
+        <v>0</v>
+      </c>
+      <c r="F9" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" s="2" ht="16.75" customHeight="1">
+      <c r="A10" s="9">
         <v>60009</v>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B10" s="3">
         <v>40002</v>
       </c>
-      <c r="C10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" ht="16.75" customHeight="1" s="2">
+      <c r="C10" s="3">
+        <v>0</v>
+      </c>
+      <c r="D10" s="3">
+        <v>0</v>
+      </c>
+      <c r="F10" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" s="2" ht="16.75" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>61001</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n">
+        <v/>
+        <is>
+          <t xml:space="preserve">61001</t>
+        </is>
+      </c>
+      <c r="B11" s="3">
         <v>31001</v>
       </c>
-      <c r="C11" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="3" t="n">
+      <c r="C11" s="3">
+        <v>1</v>
+      </c>
+      <c r="D11" s="3">
+        <v>1</v>
+      </c>
+      <c r="E11" s="3">
         <v>30001</v>
       </c>
-      <c r="F11" s="3" t="n">
+      <c r="F11" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>61001a</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n">
+        <v/>
+        <is>
+          <t xml:space="preserve">61001a</t>
+        </is>
+      </c>
+      <c r="B12" s="3">
         <v>31001</v>
       </c>
-      <c r="C12" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="3" t="n">
+      <c r="C12" s="3">
+        <v>1</v>
+      </c>
+      <c r="D12" s="3">
+        <v>1</v>
+      </c>
+      <c r="E12" s="3">
         <v>30001</v>
       </c>
-      <c r="F12" s="3" t="n">
+      <c r="F12" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="19" ht="16.75" customHeight="1" s="2"/>
+    <row r="13" s="2" ht="16.75" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <v/>
+        <is>
+          <t xml:space="preserve">61002</t>
+        </is>
+      </c>
+      <c r="B13" s="3">
+        <v>31002</v>
+      </c>
+      <c r="C13" s="3">
+        <v>1</v>
+      </c>
+      <c r="D13" s="3">
+        <v>1</v>
+      </c>
+      <c r="E13" s="3">
+        <v>30002</v>
+      </c>
+      <c r="F13" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" s="2" ht="16.75" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <v/>
+        <is>
+          <t xml:space="preserve">61003</t>
+        </is>
+      </c>
+      <c r="B14" s="3">
+        <v>31003</v>
+      </c>
+      <c r="C14" s="3">
+        <v>1</v>
+      </c>
+      <c r="D14" s="3">
+        <v>1</v>
+      </c>
+      <c r="E14" s="3">
+        <v>30003</v>
+      </c>
+      <c r="F14" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" s="2" ht="16.75" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <v/>
+        <is>
+          <t xml:space="preserve">61004</t>
+        </is>
+      </c>
+      <c r="B15" s="3">
+        <v>31004</v>
+      </c>
+      <c r="C15" s="3">
+        <v>1</v>
+      </c>
+      <c r="D15" s="3">
+        <v>1</v>
+      </c>
+      <c r="E15" s="3">
+        <v>30004</v>
+      </c>
+      <c r="F15" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" s="2" ht="16.75" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <v/>
+        <is>
+          <t xml:space="preserve">61005</t>
+        </is>
+      </c>
+      <c r="B16" s="3">
+        <v>31005</v>
+      </c>
+      <c r="C16" s="3">
+        <v>1</v>
+      </c>
+      <c r="D16" s="3">
+        <v>1</v>
+      </c>
+      <c r="E16" s="3">
+        <v>30005</v>
+      </c>
+      <c r="F16" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" s="2" ht="16.75" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <v/>
+        <is>
+          <t xml:space="preserve">61005a</t>
+        </is>
+      </c>
+      <c r="B17" s="3">
+        <v>31005</v>
+      </c>
+      <c r="C17" s="3">
+        <v>1</v>
+      </c>
+      <c r="D17" s="3">
+        <v>1</v>
+      </c>
+      <c r="E17" s="3">
+        <v>30005</v>
+      </c>
+      <c r="F17" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" s="2" ht="16.75" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <v/>
+        <is>
+          <t xml:space="preserve">61006</t>
+        </is>
+      </c>
+      <c r="B18" s="3">
+        <v>31006</v>
+      </c>
+      <c r="C18" s="3">
+        <v>1</v>
+      </c>
+      <c r="D18" s="3">
+        <v>1</v>
+      </c>
+      <c r="E18" s="3">
+        <v>30006</v>
+      </c>
+      <c r="F18" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" s="2" ht="16.75" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <v/>
+        <is>
+          <t xml:space="preserve">61006a</t>
+        </is>
+      </c>
+      <c r="B19" s="3">
+        <v>31006</v>
+      </c>
+      <c r="C19" s="3">
+        <v>1</v>
+      </c>
+      <c r="D19" s="3">
+        <v>1</v>
+      </c>
+      <c r="E19" s="3">
+        <v>30006</v>
+      </c>
+      <c r="F19" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" s="2" ht="16.75" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <v/>
+        <is>
+          <t xml:space="preserve">61007</t>
+        </is>
+      </c>
+      <c r="B20" s="3">
+        <v>31007</v>
+      </c>
+      <c r="C20" s="3">
+        <v>1</v>
+      </c>
+      <c r="D20" s="3">
+        <v>1</v>
+      </c>
+      <c r="E20" s="3">
+        <v>30007</v>
+      </c>
+      <c r="F20" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" s="2" ht="16.75" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <v/>
+        <is>
+          <t xml:space="preserve">62001</t>
+        </is>
+      </c>
+      <c r="B21" s="3">
+        <v>42001</v>
+      </c>
+      <c r="C21" s="3">
+        <v>1</v>
+      </c>
+      <c r="D21" s="3">
+        <v>1</v>
+      </c>
+      <c r="E21" s="3">
+        <v>40001</v>
+      </c>
+      <c r="F21" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" s="2" ht="16.75" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <v/>
+        <is>
+          <t xml:space="preserve">62001a</t>
+        </is>
+      </c>
+      <c r="B22" s="3">
+        <v>42001</v>
+      </c>
+      <c r="C22" s="3">
+        <v>1</v>
+      </c>
+      <c r="D22" s="3">
+        <v>1</v>
+      </c>
+      <c r="E22" s="3">
+        <v>40001</v>
+      </c>
+      <c r="F22" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" s="2" ht="16.75" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <v/>
+        <is>
+          <t xml:space="preserve">62002</t>
+        </is>
+      </c>
+      <c r="B23" s="3">
+        <v>42002</v>
+      </c>
+      <c r="C23" s="3">
+        <v>1</v>
+      </c>
+      <c r="D23" s="3">
+        <v>1</v>
+      </c>
+      <c r="E23" s="3">
+        <v>40002</v>
+      </c>
+      <c r="F23" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" s="2" ht="16.75" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <v/>
+        <is>
+          <t xml:space="preserve">62002a</t>
+        </is>
+      </c>
+      <c r="B24" s="3">
+        <v>42002</v>
+      </c>
+      <c r="C24" s="3">
+        <v>1</v>
+      </c>
+      <c r="D24" s="3">
+        <v>1</v>
+      </c>
+      <c r="E24" s="3">
+        <v>40002</v>
+      </c>
+      <c r="F24" s="3">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="0"/>
+  <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet2">
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.4"/>
   <cols>
-    <col width="10" customWidth="1" style="2" min="1" max="1"/>
-    <col width="13.92578125" customWidth="1" style="2" min="2" max="2"/>
-    <col width="26.85546875" customWidth="1" style="2" min="3" max="3"/>
-    <col width="24.28515625" customWidth="1" style="2" min="4" max="4"/>
-    <col width="13.78515625" customWidth="1" style="2" min="5" max="5"/>
+    <col min="1" max="1" width="10" style="2" customWidth="1"/>
+    <col min="2" max="2" width="13.92578125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="26.85546875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="13.78515625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>id</t>
+        <v>id</v>
+        <is>
+          <t xml:space="preserve">id</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>target_train_id</t>
+        <v>target_train_id</v>
+        <is>
+          <t xml:space="preserve">target_train_id</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>weighted_upgrades</t>
+        <v>weighted_upgrades</v>
+        <is>
+          <t xml:space="preserve">weighted_upgrades</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>weight</t>
+        <v>weight</v>
+        <is>
+          <t xml:space="preserve">weight</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>upgrade_weight</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="16.75" customHeight="1" s="2">
-      <c r="A2" s="7" t="n">
+        <v>upgrade_weight</v>
+        <is>
+          <t xml:space="preserve">upgrade_weight</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" s="2" ht="16.75" customHeight="1">
+      <c r="A2" s="7">
         <v>70001</v>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="3">
         <v>30001</v>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="C2" s="3">
         <v>90001</v>
       </c>
-      <c r="D2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" s="3" t="n">
+      <c r="D2" s="3">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3">
         <v>100</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="n">
+      <c r="A3" s="8">
         <v>70002</v>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="3">
         <v>30002</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" s="3">
         <v>90002</v>
       </c>
-      <c r="D3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3" t="n">
+      <c r="D3" s="3">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="n">
+      <c r="A4" s="8">
         <v>70003</v>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="3">
         <v>30003</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" s="3">
         <v>90003</v>
       </c>
-      <c r="D4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3" t="n">
+      <c r="D4" s="3">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="n">
+      <c r="A5" s="8">
         <v>70004</v>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="3">
         <v>30004</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5" s="3">
         <v>90004</v>
       </c>
-      <c r="D5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3" t="n">
+      <c r="D5" s="3">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="n">
+      <c r="A6" s="8">
         <v>70005</v>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="3">
         <v>30005</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="3">
         <v>90005</v>
       </c>
-      <c r="D6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="3" t="n">
+      <c r="D6" s="3">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n">
+      <c r="A7" s="8">
         <v>70006</v>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" s="3">
         <v>30006</v>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" s="3">
         <v>90006</v>
       </c>
-      <c r="D7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3" t="n">
+      <c r="D7" s="3">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="n">
+      <c r="A8" s="8">
         <v>70007</v>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" s="3">
         <v>30007</v>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C8" s="3">
         <v>90007</v>
       </c>
-      <c r="D8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="3" t="n">
+      <c r="D8" s="3">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="n">
+      <c r="A9" s="8">
         <v>70008</v>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B9" s="3">
         <v>40001</v>
       </c>
-      <c r="C9" s="3" t="n">
+      <c r="C9" s="3">
         <v>100001</v>
       </c>
-      <c r="D9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="3" t="n">
+      <c r="D9" s="3">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="n">
+      <c r="A10" s="8">
         <v>70009</v>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B10" s="3">
         <v>40002</v>
       </c>
-      <c r="C10" s="3" t="n">
+      <c r="C10" s="3">
         <v>100002</v>
       </c>
-      <c r="D10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="3" t="n">
+      <c r="D10" s="3">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="n"/>
+      <c r="A11" s="8">
+        <v>70010</v>
+      </c>
+      <c r="B11" s="3">
+        <v>31004</v>
+      </c>
+      <c r="C11" s="3">
+        <v>90008</v>
+      </c>
+      <c r="D11" s="3">
+        <v>1</v>
+      </c>
+      <c r="E11" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="n"/>
+      <c r="A12" s="8">
+        <v>70011</v>
+      </c>
+      <c r="B12" s="3">
+        <v>31004</v>
+      </c>
+      <c r="C12" s="3">
+        <v>90009</v>
+      </c>
+      <c r="D12" s="3">
+        <v>1</v>
+      </c>
+      <c r="E12" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="n"/>
+      <c r="A13" s="8"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="n"/>
+      <c r="A14" s="8"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="n"/>
-    </row>
-    <row r="16" ht="16.75" customHeight="1" s="2">
-      <c r="A16" s="9" t="n"/>
+      <c r="A15" s="8"/>
+    </row>
+    <row r="16" s="2" ht="16.75" customHeight="1">
+      <c r="A16" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="0"/>
+  <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>